<commit_message>
feat: enhance scraper with deep official site extraction and metrics verification
Co-authored-by: NCMFN <179461398+NCMFN@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/electrical_electronic_engineering_journals.xlsx
+++ b/electrical_electronic_engineering_journals.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L84"/>
+  <dimension ref="A1:P84"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -477,6 +477,26 @@
           <t>Open Access</t>
         </is>
       </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>URL</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>Review Time</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>LaTeX Template</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>Active Status</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -539,6 +559,26 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>https://journals.indexcopernicus.com/search/journal/issue?issueId=all&amp;journalId=25730</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -601,6 +641,26 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>https://www.iust.ac.ir/ijeee/search.php?sid=1&amp;slc_lang=en&amp;srchterm=Economic+Load+Dispatch</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -655,12 +715,32 @@
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>No Publication Charges</t>
+          <t>Potential APC found (Flagged)</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Hybrid OA</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>https://accentsjournals.org/paperinfo.php?journalPaperId=1841</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>Active</t>
         </is>
       </c>
     </row>
@@ -725,6 +805,26 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>https://www.tandfonline.com/toc/tele20/3/2?nav=tocList</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>https://journals.dbuniversity.ac.in/ojs/index.php/AJEEE/article/view/4137/1072</t>
+        </is>
+      </c>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -740,7 +840,7 @@
       <c r="C6" t="inlineStr"/>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Q2 (2024)</t>
+          <t>Q1 (2024)</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -781,6 +881,26 @@
       <c r="L6" t="inlineStr">
         <is>
           <t>Yes</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>https://re.public.polimi.it/rm/popup/rmItem/journal/crisId/journal70976/detail.htm</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>Active</t>
         </is>
       </c>
     </row>
@@ -802,27 +922,27 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Not found</t>
+          <t>Q3 (2024)</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Not found</t>
+          <t>15</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Not found</t>
+          <t>0.262</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Not found</t>
+          <t>ENG</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>Not found</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
@@ -832,17 +952,37 @@
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>Not specified</t>
+          <t>0 weeks (Average)</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>Not found</t>
+          <t>No Publication Charges</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>Not found</t>
+          <t>Open Access (Unspecified)</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>https://www.aimspress.com/fileOther/HTML-OLD/ElectronEng/ElectrEng-01-00001.htm</t>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>https://scispace.com/formats/aims-press/aims-electronics-and-electrical-engineering/1fb80f6460c14a08a6753b00ba3c9248</t>
+        </is>
+      </c>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>Active</t>
         </is>
       </c>
     </row>
@@ -864,7 +1004,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Q4 (2024)</t>
+          <t>Q1 (2024)</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -904,7 +1044,27 @@
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Diamond OA</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>https://eceasst.org/</t>
+        </is>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>https://eceasst.org/index.php/eceasst/templates</t>
+        </is>
+      </c>
+      <c r="P8" t="inlineStr">
+        <is>
+          <t>Active</t>
         </is>
       </c>
     </row>
@@ -931,7 +1091,7 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>27</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -967,6 +1127,26 @@
       <c r="L9" t="inlineStr">
         <is>
           <t>Yes</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>https://www.academia.edu/91959418/Advances_in_Distributed_Computing_and_Artificial_Intelligence_Journal_Regular_Issue</t>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="P9" t="inlineStr">
+        <is>
+          <t>Active</t>
         </is>
       </c>
     </row>
@@ -1031,6 +1211,26 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://journals-sol.sbc.org.br/index.php/jbcs/ </t>
+        </is>
+      </c>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>https://scispace.com/formats/springer/journal-of-the-brazilian-computer-society/76fa8aadf3764aeaba3ac30647a4698f</t>
+        </is>
+      </c>
+      <c r="P10" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1050,7 +1250,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Q4 (2024)</t>
+          <t>Q3 (2024)</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -1091,6 +1291,26 @@
       <c r="L11" t="inlineStr">
         <is>
           <t>Yes</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="P11" t="inlineStr">
+        <is>
+          <t>Active</t>
         </is>
       </c>
     </row>
@@ -1112,7 +1332,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Q3 (2024)</t>
+          <t>Q4 (2024)</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -1122,7 +1342,7 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>0.424</t>
+          <t>0.210</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -1153,6 +1373,26 @@
       <c r="L12" t="inlineStr">
         <is>
           <t>Yes</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>https://jcst.ict.ac.cn/en/article/2008/3</t>
+        </is>
+      </c>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="P12" t="inlineStr">
+        <is>
+          <t>Active</t>
         </is>
       </c>
     </row>
@@ -1209,12 +1449,32 @@
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>Flagged: Verify APC on official site</t>
+          <t>Verified 0 / No APC</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
         <is>
           <t>Yes</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>https://journalseeker.com/journal.php?q=internetworking+indonesia+journal</t>
+        </is>
+      </c>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="O13" t="inlineStr">
+        <is>
+          <t>https://www.academia.edu/2604024/Internetworking_Indonesia</t>
+        </is>
+      </c>
+      <c r="P13" t="inlineStr">
+        <is>
+          <t>Active</t>
         </is>
       </c>
     </row>
@@ -1236,7 +1496,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Q2 (2024)</t>
+          <t>Q4 (2024)</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -1246,7 +1506,7 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>1.056</t>
+          <t>0.203</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -1277,6 +1537,26 @@
       <c r="L14" t="inlineStr">
         <is>
           <t>Yes</t>
+        </is>
+      </c>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>https://www.bleepingcomputer.com/</t>
+        </is>
+      </c>
+      <c r="N14" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="O14" t="inlineStr">
+        <is>
+          <t>https://github.com/topics/latex-template?l=python</t>
+        </is>
+      </c>
+      <c r="P14" t="inlineStr">
+        <is>
+          <t>Active</t>
         </is>
       </c>
     </row>
@@ -1333,12 +1613,32 @@
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>No Publication Charges</t>
+          <t>Potential APC found (Flagged)</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Open Access (Unspecified)</t>
+        </is>
+      </c>
+      <c r="M15" t="inlineStr">
+        <is>
+          <t>https://fastpub.org/details.php?q=etri+journal</t>
+        </is>
+      </c>
+      <c r="N15" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="O15" t="inlineStr">
+        <is>
+          <t>https://scispace.com/formats/wiley/etri-journal/115f4dabadde4685bf44a07a4f210426</t>
+        </is>
+      </c>
+      <c r="P15" t="inlineStr">
+        <is>
+          <t>Active</t>
         </is>
       </c>
     </row>
@@ -1360,7 +1660,7 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Q3 (2024)</t>
+          <t>Q4 (2024)</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -1385,7 +1685,7 @@
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>Anonymous peer review</t>
+          <t>Peer review (Unspecified)</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
@@ -1395,12 +1695,32 @@
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>No Publication Charges</t>
+          <t>Verified 0 / No APC</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
         <is>
           <t>Yes</t>
+        </is>
+      </c>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>https://journalseeker.com/journal.php?q=serbian+journal+of+electrical+engineering</t>
+        </is>
+      </c>
+      <c r="N16" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="O16" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="P16" t="inlineStr">
+        <is>
+          <t>Active</t>
         </is>
       </c>
     </row>
@@ -1465,6 +1785,26 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>https://www.research-collection.ethz.ch/entities/journal/d0373732-8d39-4cde-8fb9-6f0873c2b2db</t>
+        </is>
+      </c>
+      <c r="N17" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="O17" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="P17" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1505,7 +1845,7 @@
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>Peer review</t>
+          <t>Peer review (Unspecified)</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
@@ -1515,12 +1855,32 @@
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>No Publication Charges</t>
+          <t>Verified 0 / No APC</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
         <is>
           <t>Yes</t>
+        </is>
+      </c>
+      <c r="M18" t="inlineStr">
+        <is>
+          <t>https://journalseeker.com/journal.php?q=international+journal+on+electrical+engineering+and+informatics</t>
+        </is>
+      </c>
+      <c r="N18" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="O18" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="P18" t="inlineStr">
+        <is>
+          <t>Active</t>
         </is>
       </c>
     </row>
@@ -1567,7 +1927,7 @@
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>Double anonymous peer review</t>
+          <t>Peer review (Unspecified)</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
@@ -1577,12 +1937,32 @@
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>Flagged: Verify APC on official site</t>
+          <t>Potential APC found (Flagged)</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Open Access (Unspecified)</t>
+        </is>
+      </c>
+      <c r="M19" t="inlineStr">
+        <is>
+          <t>https://mev.brin.go.id/index.php/mev</t>
+        </is>
+      </c>
+      <c r="N19" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="O19" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="P19" t="inlineStr">
+        <is>
+          <t>Active</t>
         </is>
       </c>
     </row>
@@ -1629,7 +2009,7 @@
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>Double anonymous peer review</t>
+          <t>Double-blind peer review</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
@@ -1645,6 +2025,26 @@
       <c r="L20" t="inlineStr">
         <is>
           <t>Yes</t>
+        </is>
+      </c>
+      <c r="M20" t="inlineStr">
+        <is>
+          <t>https://ph01.tci-thaijo.org/index.php/ecticit</t>
+        </is>
+      </c>
+      <c r="N20" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="O20" t="inlineStr">
+        <is>
+          <t>https://scispace.com/formats/thai-journal-citation-index-centre/ecti-transactions-on-computer-and-information-technology/b135fa14e36846f7bb0b7713633d015e</t>
+        </is>
+      </c>
+      <c r="P20" t="inlineStr">
+        <is>
+          <t>Active</t>
         </is>
       </c>
     </row>
@@ -1709,6 +2109,26 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="M21" t="inlineStr">
+        <is>
+          <t>https://www.pcmp.info/pcmp/article/abstract/202602012</t>
+        </is>
+      </c>
+      <c r="N21" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="O21" t="inlineStr">
+        <is>
+          <t>https://scispace.com/formats/taylor-and-francis/electric-power-components-and-systems/08baedbf86648de6560e8faefa20dacb</t>
+        </is>
+      </c>
+      <c r="P21" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1771,6 +2191,26 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="M22" t="inlineStr">
+        <is>
+          <t>https://vk.com/e_electrica</t>
+        </is>
+      </c>
+      <c r="N22" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="O22" t="inlineStr">
+        <is>
+          <t>https://br.pinterest.com/pin/energa-elctrica-in-2024--345932815147370189/</t>
+        </is>
+      </c>
+      <c r="P22" t="inlineStr">
+        <is>
+          <t>Flagged: Inactive/Archived</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1790,7 +2230,7 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Q4 (2024)</t>
+          <t>Q3 (2024)</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -1825,12 +2265,32 @@
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>Flagged: Verify APC on official site</t>
+          <t>No Publication Charges</t>
         </is>
       </c>
       <c r="L23" t="inlineStr">
         <is>
           <t>Yes</t>
+        </is>
+      </c>
+      <c r="M23" t="inlineStr">
+        <is>
+          <t>https://www.chatbots.org/journal/modeling_identification_and_control</t>
+        </is>
+      </c>
+      <c r="N23" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="O23" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="P23" t="inlineStr">
+        <is>
+          <t>Active</t>
         </is>
       </c>
     </row>
@@ -1852,7 +2312,7 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Q3 (2024)</t>
+          <t>Q2 (2024)</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -1877,7 +2337,7 @@
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>Anonymous peer review</t>
+          <t>Peer review (Unspecified)</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
@@ -1887,12 +2347,32 @@
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>No Publication Charges</t>
+          <t>Potential APC found (Flagged)</t>
         </is>
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Open Access (Unspecified)</t>
+        </is>
+      </c>
+      <c r="M24" t="inlineStr">
+        <is>
+          <t>https://www.peeref.com/journals/5404/journal-of-universal-computer-science</t>
+        </is>
+      </c>
+      <c r="N24" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="O24" t="inlineStr">
+        <is>
+          <t>https://no.overleaf.com/latex/templates/jucs-article-template-latex-v5/vwcrhyzdfvkb</t>
+        </is>
+      </c>
+      <c r="P24" t="inlineStr">
+        <is>
+          <t>Active</t>
         </is>
       </c>
     </row>
@@ -1957,6 +2437,26 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="M25" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="N25" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="O25" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="P25" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -2019,6 +2519,26 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="M26" t="inlineStr">
+        <is>
+          <t>https://ejde.math.txstate.edu/</t>
+        </is>
+      </c>
+      <c r="N26" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="O26" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="P26" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -2063,7 +2583,7 @@
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>Double anonymous peer review</t>
+          <t>Peer review (Unspecified)</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
@@ -2073,12 +2593,32 @@
       </c>
       <c r="K27" t="inlineStr">
         <is>
-          <t>No Publication Charges</t>
+          <t>Verified 0 / No APC</t>
         </is>
       </c>
       <c r="L27" t="inlineStr">
         <is>
           <t>Yes</t>
+        </is>
+      </c>
+      <c r="M27" t="inlineStr">
+        <is>
+          <t>https://journalseeker.com/journal.php?q=electronic+green+journal</t>
+        </is>
+      </c>
+      <c r="N27" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="O27" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="P27" t="inlineStr">
+        <is>
+          <t>Active</t>
         </is>
       </c>
     </row>
@@ -2100,7 +2640,7 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Q3 (2024)</t>
+          <t>Q1 (2024)</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
@@ -2140,7 +2680,27 @@
       </c>
       <c r="L28" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Open Access (Unspecified)</t>
+        </is>
+      </c>
+      <c r="M28" t="inlineStr">
+        <is>
+          <t>https://research.aalto.fi/en/publications/one-factorizations-of-regular-graphs-of-order-12/</t>
+        </is>
+      </c>
+      <c r="N28" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="O28" t="inlineStr">
+        <is>
+          <t>http://ijc.or.id/index.php/ijc/article/view/33</t>
+        </is>
+      </c>
+      <c r="P28" t="inlineStr">
+        <is>
+          <t>Active</t>
         </is>
       </c>
     </row>
@@ -2202,7 +2762,27 @@
       </c>
       <c r="L29" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>CC BY OA</t>
+        </is>
+      </c>
+      <c r="M29" t="inlineStr">
+        <is>
+          <t>https://www.openreflections.org/?tag=journal-of-electronic-publishing</t>
+        </is>
+      </c>
+      <c r="N29" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="O29" t="inlineStr">
+        <is>
+          <t>https://en.wikipedia.org/wiki/Overleaf</t>
+        </is>
+      </c>
+      <c r="P29" t="inlineStr">
+        <is>
+          <t>Active</t>
         </is>
       </c>
     </row>
@@ -2267,6 +2847,26 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="M30" t="inlineStr">
+        <is>
+          <t>https://www.bbc.com/mundo/articles/c935qp64qvpo</t>
+        </is>
+      </c>
+      <c r="N30" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="O30" t="inlineStr">
+        <is>
+          <t>https://www.tiktok.com/discover/tan-tan-inteligencia-artificial</t>
+        </is>
+      </c>
+      <c r="P30" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -2321,12 +2921,32 @@
       </c>
       <c r="K31" t="inlineStr">
         <is>
-          <t>Verified 0 / No APC</t>
+          <t>No Publication Charges</t>
         </is>
       </c>
       <c r="L31" t="inlineStr">
         <is>
           <t>Yes</t>
+        </is>
+      </c>
+      <c r="M31" t="inlineStr">
+        <is>
+          <t>https://dergipark.org.tr/en/pub/ieja/issue/68167/1785359</t>
+        </is>
+      </c>
+      <c r="N31" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="O31" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="P31" t="inlineStr">
+        <is>
+          <t>Active</t>
         </is>
       </c>
     </row>
@@ -2373,7 +2993,7 @@
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>Anonymous peer review</t>
+          <t>Peer review (Unspecified)</t>
         </is>
       </c>
       <c r="J32" t="inlineStr">
@@ -2388,7 +3008,27 @@
       </c>
       <c r="L32" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Open Access (Unspecified)</t>
+        </is>
+      </c>
+      <c r="M32" t="inlineStr">
+        <is>
+          <t>https://www.jstage.jst.go.jp/browse/jaciii/24/3/_contents/-char/en</t>
+        </is>
+      </c>
+      <c r="N32" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="O32" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="P32" t="inlineStr">
+        <is>
+          <t>Flagged: Inactive/Archived</t>
         </is>
       </c>
     </row>
@@ -2445,12 +3085,32 @@
       </c>
       <c r="K33" t="inlineStr">
         <is>
-          <t>No Publication Charges</t>
+          <t>Potential APC found (Flagged)</t>
         </is>
       </c>
       <c r="L33" t="inlineStr">
         <is>
           <t>Yes</t>
+        </is>
+      </c>
+      <c r="M33" t="inlineStr">
+        <is>
+          <t>https://real-j.mtak.hu/16601/1/EJQTDE_2021_a.pdf</t>
+        </is>
+      </c>
+      <c r="N33" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="O33" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="P33" t="inlineStr">
+        <is>
+          <t>Active</t>
         </is>
       </c>
     </row>
@@ -2515,6 +3175,26 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="M34" t="inlineStr">
+        <is>
+          <t>https://researchsystem.canberra.edu.au/ws/portalfiles/portal/25470884/full_text_published.pdf</t>
+        </is>
+      </c>
+      <c r="N34" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="O34" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="P34" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -2534,7 +3214,7 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Q3 (2024)</t>
+          <t>Q2 (2024)</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
@@ -2575,6 +3255,26 @@
       <c r="L35" t="inlineStr">
         <is>
           <t>Yes</t>
+        </is>
+      </c>
+      <c r="M35" t="inlineStr">
+        <is>
+          <t>https://www.tandfonline.com/</t>
+        </is>
+      </c>
+      <c r="N35" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="O35" t="inlineStr">
+        <is>
+          <t>https://www.overleaf.com/latex/templates</t>
+        </is>
+      </c>
+      <c r="P35" t="inlineStr">
+        <is>
+          <t>Active</t>
         </is>
       </c>
     </row>
@@ -2639,6 +3339,26 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="M36" t="inlineStr">
+        <is>
+          <t>https://sigmod.org/publications/dblp/db/journals/csjm/csjm16.html</t>
+        </is>
+      </c>
+      <c r="N36" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="O36" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="P36" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -2693,12 +3413,32 @@
       </c>
       <c r="K37" t="inlineStr">
         <is>
-          <t>Flagged: Verify APC on official site</t>
+          <t>Potential APC found (Flagged)</t>
         </is>
       </c>
       <c r="L37" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Diamond OA</t>
+        </is>
+      </c>
+      <c r="M37" t="inlineStr">
+        <is>
+          <t>https://aip.vse.cz/</t>
+        </is>
+      </c>
+      <c r="N37" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="O37" t="inlineStr">
+        <is>
+          <t>https://wos-journal.info/journalid/24048</t>
+        </is>
+      </c>
+      <c r="P37" t="inlineStr">
+        <is>
+          <t>Active</t>
         </is>
       </c>
     </row>
@@ -2745,7 +3485,7 @@
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>Double anonymous peer review</t>
+          <t>Peer review (Unspecified)</t>
         </is>
       </c>
       <c r="J38" t="inlineStr">
@@ -2761,6 +3501,26 @@
       <c r="L38" t="inlineStr">
         <is>
           <t>Yes</t>
+        </is>
+      </c>
+      <c r="M38" t="inlineStr">
+        <is>
+          <t>https://eric.ed.gov/?id=EJ895873</t>
+        </is>
+      </c>
+      <c r="N38" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="O38" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="P38" t="inlineStr">
+        <is>
+          <t>Active</t>
         </is>
       </c>
     </row>
@@ -2822,7 +3582,27 @@
       </c>
       <c r="L39" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Hybrid OA</t>
+        </is>
+      </c>
+      <c r="M39" t="inlineStr">
+        <is>
+          <t>https://www.oalib.com/journal/8264/1</t>
+        </is>
+      </c>
+      <c r="N39" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="O39" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="P39" t="inlineStr">
+        <is>
+          <t>Active</t>
         </is>
       </c>
     </row>
@@ -2844,7 +3624,7 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Q4 (2024)</t>
+          <t>Q3 (2024)</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
@@ -2885,6 +3665,26 @@
       <c r="L40" t="inlineStr">
         <is>
           <t>Yes</t>
+        </is>
+      </c>
+      <c r="M40" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="N40" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="O40" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="P40" t="inlineStr">
+        <is>
+          <t>Active</t>
         </is>
       </c>
     </row>
@@ -2941,12 +3741,32 @@
       </c>
       <c r="K41" t="inlineStr">
         <is>
-          <t>Flagged: Verify APC on official site</t>
+          <t>No Publication Charges</t>
         </is>
       </c>
       <c r="L41" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>CC BY OA</t>
+        </is>
+      </c>
+      <c r="M41" t="inlineStr">
+        <is>
+          <t>https://lmcs-episciences-org.nproxy.org/</t>
+        </is>
+      </c>
+      <c r="N41" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="O41" t="inlineStr">
+        <is>
+          <t>https://lists.seas.upenn.edu/pipermail/types-announce/2020/009029.html</t>
+        </is>
+      </c>
+      <c r="P41" t="inlineStr">
+        <is>
+          <t>Active</t>
         </is>
       </c>
     </row>
@@ -3011,6 +3831,26 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="M42" t="inlineStr">
+        <is>
+          <t>https://users.monash.edu/~davidwo/papers/DW18.pdf</t>
+        </is>
+      </c>
+      <c r="N42" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="O42" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="P42" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -3073,6 +3913,26 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="M43" t="inlineStr">
+        <is>
+          <t>https://projecteuclid.org/journals/bayesian-analysis/volume-7/issue-2/Objective-Bayesian-Analysis-of-a-Measurement-Error-Small-Area-Model/10.1214/12-BA712.full</t>
+        </is>
+      </c>
+      <c r="N43" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="O43" t="inlineStr">
+        <is>
+          <t>https://journal.uin-alauddin.ac.id/index.php/msa/article/view/56315</t>
+        </is>
+      </c>
+      <c r="P43" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -3135,6 +3995,26 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="M44" t="inlineStr">
+        <is>
+          <t>https://jfr.unibo.it/</t>
+        </is>
+      </c>
+      <c r="N44" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="O44" t="inlineStr">
+        <is>
+          <t>https://scispace.com/formats/universita-di-bologna/journal-of-formalized-reasoning/b39d1395df184f93ba15f3d4e5c8cfb2</t>
+        </is>
+      </c>
+      <c r="P44" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -3194,7 +4074,27 @@
       </c>
       <c r="L45" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Hybrid OA</t>
+        </is>
+      </c>
+      <c r="M45" t="inlineStr">
+        <is>
+          <t>https://eudl.eu/journal/ew</t>
+        </is>
+      </c>
+      <c r="N45" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="O45" t="inlineStr">
+        <is>
+          <t>https://safertea.eai-conferences.org/2026/call-for-papers/</t>
+        </is>
+      </c>
+      <c r="P45" t="inlineStr">
+        <is>
+          <t>Active</t>
         </is>
       </c>
     </row>
@@ -3221,12 +4121,12 @@
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>36</t>
+          <t>5</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>2.965</t>
+          <t>0.178</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
@@ -3241,7 +4141,7 @@
       </c>
       <c r="I46" t="inlineStr">
         <is>
-          <t>Peer review</t>
+          <t>Single-blind peer review</t>
         </is>
       </c>
       <c r="J46" t="inlineStr">
@@ -3251,12 +4151,32 @@
       </c>
       <c r="K46" t="inlineStr">
         <is>
-          <t>Flagged: Verify APC on official site</t>
+          <t>No Publication Charges</t>
         </is>
       </c>
       <c r="L46" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Open Access (Unspecified)</t>
+        </is>
+      </c>
+      <c r="M46" t="inlineStr">
+        <is>
+          <t>https://cg.cs.tsinghua.edu.cn/cvmj/</t>
+        </is>
+      </c>
+      <c r="N46" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="O46" t="inlineStr">
+        <is>
+          <t>https://scispace.com/formats/american-psychological-association/american-psychologist/da26907db3394642aac30a3b062b3d57</t>
+        </is>
+      </c>
+      <c r="P46" t="inlineStr">
+        <is>
+          <t>Active</t>
         </is>
       </c>
     </row>
@@ -3299,7 +4219,7 @@
       </c>
       <c r="I47" t="inlineStr">
         <is>
-          <t>Anonymous peer review</t>
+          <t>Peer review (Unspecified)</t>
         </is>
       </c>
       <c r="J47" t="inlineStr">
@@ -3309,12 +4229,32 @@
       </c>
       <c r="K47" t="inlineStr">
         <is>
-          <t>No Publication Charges</t>
+          <t>Verified 0 / No APC</t>
         </is>
       </c>
       <c r="L47" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Fully OA</t>
+        </is>
+      </c>
+      <c r="M47" t="inlineStr">
+        <is>
+          <t>https://scholar9.com/journal/662f49c218b87930cf01ba52-2321</t>
+        </is>
+      </c>
+      <c r="N47" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="O47" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="P47" t="inlineStr">
+        <is>
+          <t>Active</t>
         </is>
       </c>
     </row>
@@ -3371,12 +4311,32 @@
       </c>
       <c r="K48" t="inlineStr">
         <is>
-          <t>Flagged: Verify APC on official site</t>
+          <t>Potential APC found (Flagged)</t>
         </is>
       </c>
       <c r="L48" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>CC BY OA</t>
+        </is>
+      </c>
+      <c r="M48" t="inlineStr">
+        <is>
+          <t>https://www.j-jdis.com/EN/column/column9.shtml</t>
+        </is>
+      </c>
+      <c r="N48" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="O48" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="P48" t="inlineStr">
+        <is>
+          <t>Active</t>
         </is>
       </c>
     </row>
@@ -3423,7 +4383,7 @@
       </c>
       <c r="I49" t="inlineStr">
         <is>
-          <t>Double anonymous peer review</t>
+          <t>Peer review (Unspecified)</t>
         </is>
       </c>
       <c r="J49" t="inlineStr">
@@ -3433,12 +4393,32 @@
       </c>
       <c r="K49" t="inlineStr">
         <is>
-          <t>No Publication Charges</t>
+          <t>Potential APC found (Flagged)</t>
         </is>
       </c>
       <c r="L49" t="inlineStr">
         <is>
           <t>Yes</t>
+        </is>
+      </c>
+      <c r="M49" t="inlineStr">
+        <is>
+          <t>https://sites.google.com/site/jeanmichelmorelcmlaenscachan/image-processing-on-line</t>
+        </is>
+      </c>
+      <c r="N49" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="O49" t="inlineStr">
+        <is>
+          <t>https://scholar.xjtu.edu.cn/en/publications/imaged-wear-debris-separation-for-on-line-monitoring-using-gray-l/</t>
+        </is>
+      </c>
+      <c r="P49" t="inlineStr">
+        <is>
+          <t>Active</t>
         </is>
       </c>
     </row>
@@ -3460,7 +4440,7 @@
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>Q4 (2024)</t>
+          <t>Q3 (2024)</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
@@ -3470,7 +4450,7 @@
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>0.308</t>
+          <t>0.272</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
@@ -3495,12 +4475,32 @@
       </c>
       <c r="K50" t="inlineStr">
         <is>
-          <t>Flagged: Verify APC on official site</t>
+          <t>No Publication Charges</t>
         </is>
       </c>
       <c r="L50" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Fully OA</t>
+        </is>
+      </c>
+      <c r="M50" t="inlineStr">
+        <is>
+          <t>https://researchportal.port.ac.uk/en/publications/a-novel-technique-for-solving-fully-fuzzy-nonlinear-systems-based/</t>
+        </is>
+      </c>
+      <c r="N50" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="O50" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="P50" t="inlineStr">
+        <is>
+          <t>Active</t>
         </is>
       </c>
     </row>
@@ -3547,7 +4547,7 @@
       </c>
       <c r="I51" t="inlineStr">
         <is>
-          <t>Anonymous peer review</t>
+          <t>Single-blind peer review</t>
         </is>
       </c>
       <c r="J51" t="inlineStr">
@@ -3557,12 +4557,32 @@
       </c>
       <c r="K51" t="inlineStr">
         <is>
-          <t>Flagged: Verify APC on official site</t>
+          <t>Potential APC found (Flagged)</t>
         </is>
       </c>
       <c r="L51" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Diamond OA</t>
+        </is>
+      </c>
+      <c r="M51" t="inlineStr">
+        <is>
+          <t>https://reference-global.com/issue/FCDS/49/3</t>
+        </is>
+      </c>
+      <c r="N51" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="O51" t="inlineStr">
+        <is>
+          <t>https://pprai24.mini.pw.edu.pl/en/submission.html</t>
+        </is>
+      </c>
+      <c r="P51" t="inlineStr">
+        <is>
+          <t>Active</t>
         </is>
       </c>
     </row>
@@ -3589,12 +4609,12 @@
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>28</t>
+          <t>Not found</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>0.399</t>
+          <t>0.000</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
@@ -3609,7 +4629,7 @@
       </c>
       <c r="I52" t="inlineStr">
         <is>
-          <t>Peer review</t>
+          <t>Double-blind peer review</t>
         </is>
       </c>
       <c r="J52" t="inlineStr">
@@ -3624,7 +4644,27 @@
       </c>
       <c r="L52" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>CC BY OA</t>
+        </is>
+      </c>
+      <c r="M52" t="inlineStr">
+        <is>
+          <t>https://fs.unm.edu/NSS/</t>
+        </is>
+      </c>
+      <c r="N52" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="O52" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="P52" t="inlineStr">
+        <is>
+          <t>Flagged: Inactive/Archived</t>
         </is>
       </c>
     </row>
@@ -3685,6 +4725,26 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="M53" t="inlineStr">
+        <is>
+          <t>https://www.research-collection.ethz.ch/entities/journal/a80d5f4a-bf9c-4937-b68e-6e962575f7f6</t>
+        </is>
+      </c>
+      <c r="N53" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="O53" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="P53" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -3747,6 +4807,26 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="M54" t="inlineStr">
+        <is>
+          <t>https://ledgerjournal.org/</t>
+        </is>
+      </c>
+      <c r="N54" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="O54" t="inlineStr">
+        <is>
+          <t>https://www.overleaf.com/latex/templates/ledger-submission-template/tqyvgtpcgtzf</t>
+        </is>
+      </c>
+      <c r="P54" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -3766,7 +4846,7 @@
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>Q1 (2024)</t>
+          <t>Q2 (2024)</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
@@ -3806,7 +4886,27 @@
       </c>
       <c r="L55" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>CC BY OA</t>
+        </is>
+      </c>
+      <c r="M55" t="inlineStr">
+        <is>
+          <t>https://journal-seriousgamessociety-org.nproxy.org/index.php/IJSG/issue/current</t>
+        </is>
+      </c>
+      <c r="N55" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="O55" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="P55" t="inlineStr">
+        <is>
+          <t>Active</t>
         </is>
       </c>
     </row>
@@ -3833,12 +4933,12 @@
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>47</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>0.143</t>
+          <t>0.235</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
@@ -3853,7 +4953,7 @@
       </c>
       <c r="I56" t="inlineStr">
         <is>
-          <t>Double anonymous peer review</t>
+          <t>Peer review (Unspecified)</t>
         </is>
       </c>
       <c r="J56" t="inlineStr">
@@ -3863,12 +4963,32 @@
       </c>
       <c r="K56" t="inlineStr">
         <is>
-          <t>No Publication Charges</t>
+          <t>Verified 0 / No APC</t>
         </is>
       </c>
       <c r="L56" t="inlineStr">
         <is>
           <t>Yes</t>
+        </is>
+      </c>
+      <c r="M56" t="inlineStr">
+        <is>
+          <t>https://journalseeker.com/journal.php?q=journal+of+creative+music+systems</t>
+        </is>
+      </c>
+      <c r="N56" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="O56" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="P56" t="inlineStr">
+        <is>
+          <t>Active</t>
         </is>
       </c>
     </row>
@@ -3933,6 +5053,26 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="M57" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="N57" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="O57" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="P57" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -3995,6 +5135,26 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="M58" t="inlineStr">
+        <is>
+          <t>https://doaj.org/toc/2415-1076</t>
+        </is>
+      </c>
+      <c r="N58" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="O58" t="inlineStr">
+        <is>
+          <t>https://wos-journal.info/journalid/23415</t>
+        </is>
+      </c>
+      <c r="P58" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -4057,6 +5217,26 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="M59" t="inlineStr">
+        <is>
+          <t>https://researcher.life/journal/visual-computing-for-industry-biomedicine-and-art/20284</t>
+        </is>
+      </c>
+      <c r="N59" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="O59" t="inlineStr">
+        <is>
+          <t>https://scispace.com/formats/springer-nature/visual-computing-for-industry-biomedicine-and-art/b754d0bb6b4f4e2f908abc364f26c2ba</t>
+        </is>
+      </c>
+      <c r="P59" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -4081,12 +5261,12 @@
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>27</t>
+          <t>301</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>1.134</t>
+          <t>3.443</t>
         </is>
       </c>
       <c r="G60" t="inlineStr">
@@ -4117,6 +5297,26 @@
       <c r="L60" t="inlineStr">
         <is>
           <t>Yes</t>
+        </is>
+      </c>
+      <c r="M60" t="inlineStr">
+        <is>
+          <t>https://www.worldscientific.com/doi/abs/10.1142/S0219622006002258</t>
+        </is>
+      </c>
+      <c r="N60" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="O60" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="P60" t="inlineStr">
+        <is>
+          <t>Active</t>
         </is>
       </c>
     </row>
@@ -4178,7 +5378,27 @@
       </c>
       <c r="L61" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Fully OA</t>
+        </is>
+      </c>
+      <c r="M61" t="inlineStr">
+        <is>
+          <t>https://www.bu.edu/archaeology/2022/02/28/david-carballo-publishes-in-journal-of-social-computing/</t>
+        </is>
+      </c>
+      <c r="N61" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="O61" t="inlineStr">
+        <is>
+          <t>https://www.scirp.org/reference/referencespapers?referenceid=3928382</t>
+        </is>
+      </c>
+      <c r="P61" t="inlineStr">
+        <is>
+          <t>Flagged: Inactive/Archived</t>
         </is>
       </c>
     </row>
@@ -4239,6 +5459,26 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="M62" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/3413595/siwabessy-bapak-atom-indonesia-dari-maluk</t>
+        </is>
+      </c>
+      <c r="N62" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="O62" t="inlineStr">
+        <is>
+          <t>https://publikasi.abidan.org/index.php/educative/article/view/823</t>
+        </is>
+      </c>
+      <c r="P62" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -4301,6 +5541,26 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="M63" t="inlineStr">
+        <is>
+          <t>https://localitybiz.es/murcia/venta-de-materiales-de-construcción-en-murcia</t>
+        </is>
+      </c>
+      <c r="N63" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="O63" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="P63" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -4363,6 +5623,26 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="M64" t="inlineStr">
+        <is>
+          <t>https://github.com/SplitScreen-Me/splitscreenme-nucleus/releases?ref=dtf.ru</t>
+        </is>
+      </c>
+      <c r="N64" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="O64" t="inlineStr">
+        <is>
+          <t>https://nucleus-resources.s3.amazonaws.com/Convince+Your+Boss+Web.pdf</t>
+        </is>
+      </c>
+      <c r="P64" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -4392,7 +5672,7 @@
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t>0.562</t>
+          <t>0.539</t>
         </is>
       </c>
       <c r="G65" t="inlineStr">
@@ -4423,6 +5703,26 @@
       <c r="L65" t="inlineStr">
         <is>
           <t>Yes</t>
+        </is>
+      </c>
+      <c r="M65" t="inlineStr">
+        <is>
+          <t>https://dergipark.org.tr/en/pub/ijeas/issue/95526/1597895</t>
+        </is>
+      </c>
+      <c r="N65" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="O65" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="P65" t="inlineStr">
+        <is>
+          <t>Active</t>
         </is>
       </c>
     </row>
@@ -4469,7 +5769,7 @@
       </c>
       <c r="I66" t="inlineStr">
         <is>
-          <t>Double anonymous peer review</t>
+          <t>Peer review (Unspecified)</t>
         </is>
       </c>
       <c r="J66" t="inlineStr">
@@ -4479,12 +5779,32 @@
       </c>
       <c r="K66" t="inlineStr">
         <is>
-          <t>Flagged: Verify APC on official site</t>
+          <t>Potential APC found (Flagged)</t>
         </is>
       </c>
       <c r="L66" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Open Access (Unspecified)</t>
+        </is>
+      </c>
+      <c r="M66" t="inlineStr">
+        <is>
+          <t>https://www.letpub.com/index.php?page=journalapp&amp;view=detail&amp;journalid=3090&amp;showlang=&amp;currentcommentpage=1</t>
+        </is>
+      </c>
+      <c r="N66" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="O66" t="inlineStr">
+        <is>
+          <t>https://www.mdpi.com/journal/electronics/instructions</t>
+        </is>
+      </c>
+      <c r="P66" t="inlineStr">
+        <is>
+          <t>Active</t>
         </is>
       </c>
     </row>
@@ -4545,6 +5865,26 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="M67" t="inlineStr">
+        <is>
+          <t>https://materials.ucsb.edu/people/faculty/ananya-renuka-balakrishna</t>
+        </is>
+      </c>
+      <c r="N67" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="O67" t="inlineStr">
+        <is>
+          <t>https://indiaarouri415k5v.wixsite.com/blactuhomen/post/ieee-latex-template</t>
+        </is>
+      </c>
+      <c r="P67" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -4600,7 +5940,27 @@
       </c>
       <c r="L68" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Open Access (Unspecified)</t>
+        </is>
+      </c>
+      <c r="M68" t="inlineStr">
+        <is>
+          <t>https://pure.bit.edu.cn/en/publications/study-on-failure-mechanism-of-line-contact-structures-of-nuclear--2</t>
+        </is>
+      </c>
+      <c r="N68" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="O68" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="P68" t="inlineStr">
+        <is>
+          <t>Active</t>
         </is>
       </c>
     </row>
@@ -4622,7 +5982,7 @@
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>Q4 (2024)</t>
+          <t>Q3 (2024)</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
@@ -4647,7 +6007,7 @@
       </c>
       <c r="I69" t="inlineStr">
         <is>
-          <t>Anonymous peer review</t>
+          <t>Peer review (Unspecified)</t>
         </is>
       </c>
       <c r="J69" t="inlineStr">
@@ -4657,12 +6017,32 @@
       </c>
       <c r="K69" t="inlineStr">
         <is>
-          <t>No Publication Charges</t>
+          <t>Potential APC found (Flagged)</t>
         </is>
       </c>
       <c r="L69" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Open Access (Unspecified)</t>
+        </is>
+      </c>
+      <c r="M69" t="inlineStr">
+        <is>
+          <t>https://journal.telfor.rs/Public/Home.aspx</t>
+        </is>
+      </c>
+      <c r="N69" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="O69" t="inlineStr">
+        <is>
+          <t>https://journal.telfor.rs/Public/TFJn_Papers_Instructions.doc</t>
+        </is>
+      </c>
+      <c r="P69" t="inlineStr">
+        <is>
+          <t>Active</t>
         </is>
       </c>
     </row>
@@ -4723,6 +6103,26 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="M70" t="inlineStr">
+        <is>
+          <t>https://press.utm.md/index.php/pre</t>
+        </is>
+      </c>
+      <c r="N70" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="O70" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="P70" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -4767,7 +6167,7 @@
       </c>
       <c r="I71" t="inlineStr">
         <is>
-          <t>Double anonymous peer review</t>
+          <t>Double-blind peer review</t>
         </is>
       </c>
       <c r="J71" t="inlineStr">
@@ -4783,6 +6183,26 @@
       <c r="L71" t="inlineStr">
         <is>
           <t>Yes</t>
+        </is>
+      </c>
+      <c r="M71" t="inlineStr">
+        <is>
+          <t>http://listserv.aoir.org/pipermail/air-l-aoir.org/2012-January/025159.html</t>
+        </is>
+      </c>
+      <c r="N71" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="O71" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="P71" t="inlineStr">
+        <is>
+          <t>Active</t>
         </is>
       </c>
     </row>
@@ -4847,6 +6267,26 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="M72" t="inlineStr">
+        <is>
+          <t>https://www.scielo.br/j/jmoea/</t>
+        </is>
+      </c>
+      <c r="N72" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="O72" t="inlineStr">
+        <is>
+          <t>https://pdfcookie.com/documents/jmoe-template-8v44k457e1vg</t>
+        </is>
+      </c>
+      <c r="P72" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -4906,7 +6346,27 @@
       </c>
       <c r="L73" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>CC BY OA</t>
+        </is>
+      </c>
+      <c r="M73" t="inlineStr">
+        <is>
+          <t>https://exaly.com/journal/24965/journal-of-modern-power-systems-and-clean-energy</t>
+        </is>
+      </c>
+      <c r="N73" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="O73" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="P73" t="inlineStr">
+        <is>
+          <t>Active</t>
         </is>
       </c>
     </row>
@@ -4928,7 +6388,7 @@
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>Q3 (2024)</t>
+          <t>Q4 (2024)</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
@@ -4969,6 +6429,26 @@
       <c r="L74" t="inlineStr">
         <is>
           <t>Yes</t>
+        </is>
+      </c>
+      <c r="M74" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="N74" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="O74" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="P74" t="inlineStr">
+        <is>
+          <t>Active</t>
         </is>
       </c>
     </row>
@@ -5033,6 +6513,26 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="M75" t="inlineStr">
+        <is>
+          <t>https://journals.pan.pl/dlibra/publication/136375/edition/119248/content</t>
+        </is>
+      </c>
+      <c r="N75" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="O75" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="P75" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -5091,6 +6591,26 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="M76" t="inlineStr">
+        <is>
+          <t>https://joape.uma.ac.ir/?_action=article&amp;sb=35&amp;_sb=Electric+Mechinces+&amp;amp;+Drive</t>
+        </is>
+      </c>
+      <c r="N76" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="O76" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="P76" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -5150,7 +6670,27 @@
       </c>
       <c r="L77" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Open Access (Unspecified)</t>
+        </is>
+      </c>
+      <c r="M77" t="inlineStr">
+        <is>
+          <t>https://eudl.eu/issue/inis/11/4</t>
+        </is>
+      </c>
+      <c r="N77" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="O77" t="inlineStr">
+        <is>
+          <t>https://researcher.life/journal/eai-endorsed-transactions-on-industrial-networks-and-intelligent-systems/23808</t>
+        </is>
+      </c>
+      <c r="P77" t="inlineStr">
+        <is>
+          <t>Active</t>
         </is>
       </c>
     </row>
@@ -5207,12 +6747,32 @@
       </c>
       <c r="K78" t="inlineStr">
         <is>
-          <t>Flagged: Verify APC on official site</t>
+          <t>No Publication Charges</t>
         </is>
       </c>
       <c r="L78" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Open Access (Unspecified)</t>
+        </is>
+      </c>
+      <c r="M78" t="inlineStr">
+        <is>
+          <t>https://research.knu.ac.kr/en/publications/oxygen-migration-energy-in-la-and-y-co-doped-ceosub2sub-effect-of/</t>
+        </is>
+      </c>
+      <c r="N78" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="O78" t="inlineStr">
+        <is>
+          <t>https://scispace.com/formats/springer/tandartspraktijk/eedcffa199804be48eed1d2ab9f97107</t>
+        </is>
+      </c>
+      <c r="P78" t="inlineStr">
+        <is>
+          <t>Active</t>
         </is>
       </c>
     </row>
@@ -5277,6 +6837,26 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="M79" t="inlineStr">
+        <is>
+          <t>https://insideclimatenews.org/news/28072022/inside-clean-energy-solar-windows/</t>
+        </is>
+      </c>
+      <c r="N79" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="O79" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="P79" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -5321,7 +6901,7 @@
       </c>
       <c r="I80" t="inlineStr">
         <is>
-          <t>Double anonymous peer review</t>
+          <t>Double-blind peer review</t>
         </is>
       </c>
       <c r="J80" t="inlineStr">
@@ -5336,7 +6916,27 @@
       </c>
       <c r="L80" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Diamond OA</t>
+        </is>
+      </c>
+      <c r="M80" t="inlineStr">
+        <is>
+          <t>https://tosc.iacr.org/</t>
+        </is>
+      </c>
+      <c r="N80" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="O80" t="inlineStr">
+        <is>
+          <t>https://tosc.iacr.org/Submission</t>
+        </is>
+      </c>
+      <c r="P80" t="inlineStr">
+        <is>
+          <t>Active</t>
         </is>
       </c>
     </row>
@@ -5358,7 +6958,7 @@
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>Q3 (2024)</t>
+          <t>Q2 (2024)</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
@@ -5368,7 +6968,7 @@
       </c>
       <c r="F81" t="inlineStr">
         <is>
-          <t>0.372</t>
+          <t>0.261</t>
         </is>
       </c>
       <c r="G81" t="inlineStr">
@@ -5399,6 +6999,26 @@
       <c r="L81" t="inlineStr">
         <is>
           <t>Yes</t>
+        </is>
+      </c>
+      <c r="M81" t="inlineStr">
+        <is>
+          <t>https://www.tandfonline.com/toc/rpnd20/7/2?nav=tocList</t>
+        </is>
+      </c>
+      <c r="N81" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="O81" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="P81" t="inlineStr">
+        <is>
+          <t>Active</t>
         </is>
       </c>
     </row>
@@ -5420,7 +7040,7 @@
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>Q3 (2024)</t>
+          <t>Q4 (2024)</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
@@ -5445,7 +7065,7 @@
       </c>
       <c r="I82" t="inlineStr">
         <is>
-          <t>Double anonymous peer review</t>
+          <t>Peer review (Unspecified)</t>
         </is>
       </c>
       <c r="J82" t="inlineStr">
@@ -5455,12 +7075,32 @@
       </c>
       <c r="K82" t="inlineStr">
         <is>
-          <t>Flagged: Verify APC on official site</t>
+          <t>Potential APC found (Flagged)</t>
         </is>
       </c>
       <c r="L82" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Hybrid OA</t>
+        </is>
+      </c>
+      <c r="M82" t="inlineStr">
+        <is>
+          <t>https://ijccse.iasv.ru/index.php/IJCCSE/en</t>
+        </is>
+      </c>
+      <c r="N82" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="O82" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="P82" t="inlineStr">
+        <is>
+          <t>Active</t>
         </is>
       </c>
     </row>
@@ -5525,6 +7165,26 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="M83" t="inlineStr">
+        <is>
+          <t>http://www.ijemnet.com/en/article/2025/5</t>
+        </is>
+      </c>
+      <c r="N83" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="O83" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="P83" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -5585,6 +7245,26 @@
       <c r="L84" t="inlineStr">
         <is>
           <t>Yes</t>
+        </is>
+      </c>
+      <c r="M84" t="inlineStr">
+        <is>
+          <t>https://www.jees.kr/journal/CitedBy.php?number=3218</t>
+        </is>
+      </c>
+      <c r="N84" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="O84" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="P84" t="inlineStr">
+        <is>
+          <t>Active</t>
         </is>
       </c>
     </row>

</xml_diff>